<commit_message>
add some more photos of students
</commit_message>
<xml_diff>
--- a/stakeholders.xlsx
+++ b/stakeholders.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilliramchaudhary/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E303BE5-D72C-7342-9CF5-C66FF64EF39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B26E13-2E5B-B24F-8585-1A9B2D81B247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
+    <workbookView xWindow="12460" yWindow="880" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="61">
   <si>
     <t>Dr. Rajendra Dhoj Joshi</t>
   </si>
@@ -213,6 +213,15 @@
   </si>
   <si>
     <t>Staff</t>
+  </si>
+  <si>
+    <t>Yalamber Ingnam</t>
+  </si>
+  <si>
+    <t>Piyush Lal Shrestha</t>
+  </si>
+  <si>
+    <t>Nawaraj Luitel</t>
   </si>
 </sst>
 </file>
@@ -633,7 +642,7 @@
     </row>
     <row r="3" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="str">
-        <f t="shared" ref="A3:A53" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
+        <f t="shared" ref="A3:A56" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
         <v>0002.jpg</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1246,16 +1255,40 @@
       </c>
     </row>
     <row r="54" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="2"/>
-      <c r="C54" s="1"/>
+      <c r="A54" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0053.jpg</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="55" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="2"/>
-      <c r="C55" s="1"/>
+      <c r="A55" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0054.jpg</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="56" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="2"/>
-      <c r="C56" s="1"/>
+      <c r="A56" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0055.jpg</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="57" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2"/>

</xml_diff>

<commit_message>
add some photos of stakeholders
</commit_message>
<xml_diff>
--- a/stakeholders.xlsx
+++ b/stakeholders.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilliramchaudhary/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B26E13-2E5B-B24F-8585-1A9B2D81B247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35AB122-BB53-E646-9CD7-BB0D2114D205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12460" yWindow="880" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
+    <workbookView xWindow="9620" yWindow="820" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="64">
   <si>
     <t>Dr. Rajendra Dhoj Joshi</t>
   </si>
@@ -222,6 +222,15 @@
   </si>
   <si>
     <t>Nawaraj Luitel</t>
+  </si>
+  <si>
+    <t>Sudhin Upadhaya</t>
+  </si>
+  <si>
+    <t>Sushant Adhikari</t>
+  </si>
+  <si>
+    <t>Umesh Shahi</t>
   </si>
 </sst>
 </file>
@@ -642,7 +651,7 @@
     </row>
     <row r="3" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="str">
-        <f t="shared" ref="A3:A56" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
+        <f t="shared" ref="A3:A59" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
         <v>0002.jpg</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1291,16 +1300,40 @@
       </c>
     </row>
     <row r="57" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="2"/>
-      <c r="C57" s="1"/>
+      <c r="A57" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0056.jpg</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="58" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="2"/>
-      <c r="C58" s="1"/>
+      <c r="A58" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0057.jpg</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="59" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="2"/>
-      <c r="C59" s="1"/>
+      <c r="A59" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0058.jpg</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="60" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2"/>

</xml_diff>

<commit_message>
add some photos and info related to them
</commit_message>
<xml_diff>
--- a/stakeholders.xlsx
+++ b/stakeholders.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilliramchaudhary/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35AB122-BB53-E646-9CD7-BB0D2114D205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DEAA6B-7963-A141-A33E-EEECE93A09E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9620" yWindow="820" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
+    <workbookView xWindow="8320" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="67">
   <si>
     <t>Dr. Rajendra Dhoj Joshi</t>
   </si>
@@ -231,6 +231,15 @@
   </si>
   <si>
     <t>Umesh Shahi</t>
+  </si>
+  <si>
+    <t>Birat Dev Poudel</t>
+  </si>
+  <si>
+    <t>Binay Basenet</t>
+  </si>
+  <si>
+    <t>Sandesh Dhungana</t>
   </si>
 </sst>
 </file>
@@ -651,7 +660,7 @@
     </row>
     <row r="3" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="str">
-        <f t="shared" ref="A3:A59" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
+        <f t="shared" ref="A3:A62" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
         <v>0002.jpg</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1336,16 +1345,40 @@
       </c>
     </row>
     <row r="60" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="2"/>
-      <c r="C60" s="1"/>
+      <c r="A60" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0059.jpg</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="61" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="2"/>
-      <c r="C61" s="1"/>
+      <c r="A61" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0060.jpg</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="62" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="2"/>
-      <c r="C62" s="1"/>
+      <c r="A62" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0061.jpg</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="63" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2"/>

</xml_diff>

<commit_message>
add photo and update xcel data
</commit_message>
<xml_diff>
--- a/stakeholders.xlsx
+++ b/stakeholders.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilliramchaudhary/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DEAA6B-7963-A141-A33E-EEECE93A09E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4782398-098B-C942-A463-3ABD679D20B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8320" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="68">
   <si>
     <t>Dr. Rajendra Dhoj Joshi</t>
   </si>
@@ -224,9 +224,6 @@
     <t>Nawaraj Luitel</t>
   </si>
   <si>
-    <t>Sudhin Upadhaya</t>
-  </si>
-  <si>
     <t>Sushant Adhikari</t>
   </si>
   <si>
@@ -240,6 +237,12 @@
   </si>
   <si>
     <t>Sandesh Dhungana</t>
+  </si>
+  <si>
+    <t>Sudin Upadhaya</t>
+  </si>
+  <si>
+    <t>Hasil Silwal</t>
   </si>
 </sst>
 </file>
@@ -660,7 +663,7 @@
     </row>
     <row r="3" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="str">
-        <f t="shared" ref="A3:A62" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
+        <f t="shared" ref="A3:A63" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
         <v>0002.jpg</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1314,7 +1317,7 @@
         <v>0056.jpg</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>53</v>
@@ -1326,7 +1329,7 @@
         <v>0057.jpg</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>53</v>
@@ -1338,7 +1341,7 @@
         <v>0058.jpg</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>53</v>
@@ -1350,7 +1353,7 @@
         <v>0059.jpg</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>53</v>
@@ -1362,7 +1365,7 @@
         <v>0060.jpg</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>53</v>
@@ -1374,15 +1377,23 @@
         <v>0061.jpg</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="2"/>
-      <c r="C63" s="1"/>
+      <c r="A63" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0062.jpg</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="64" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2"/>

</xml_diff>

<commit_message>
fix: lower frame rate lagging bug has been fixed
</commit_message>
<xml_diff>
--- a/stakeholders.xlsx
+++ b/stakeholders.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilliramchaudhary/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4782398-098B-C942-A463-3ABD679D20B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88709E9D-9F4B-AC4F-8DDD-28BBF1AFD626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="69">
   <si>
     <t>Dr. Rajendra Dhoj Joshi</t>
   </si>
@@ -243,6 +243,9 @@
   </si>
   <si>
     <t>Hasil Silwal</t>
+  </si>
+  <si>
+    <t>Nisha Bhatt</t>
   </si>
 </sst>
 </file>
@@ -663,7 +666,7 @@
     </row>
     <row r="3" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="str">
-        <f t="shared" ref="A3:A63" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
+        <f t="shared" ref="A3:A64" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
         <v>0002.jpg</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1396,8 +1399,16 @@
       </c>
     </row>
     <row r="64" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="2"/>
-      <c r="C64" s="1"/>
+      <c r="A64" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0063.jpg</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="65" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2"/>

</xml_diff>

<commit_message>
add stakeholder info with photo
</commit_message>
<xml_diff>
--- a/stakeholders.xlsx
+++ b/stakeholders.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilliramchaudhary/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88709E9D-9F4B-AC4F-8DDD-28BBF1AFD626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C0D6095-838F-D34D-B80C-BB70CB2B5265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{29F8B96C-2FF4-D143-9C6F-B080B16D98CB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="70">
   <si>
     <t>Dr. Rajendra Dhoj Joshi</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t>Nisha Bhatt</t>
+  </si>
+  <si>
+    <t>Jayaram  Gautam</t>
   </si>
 </sst>
 </file>
@@ -666,7 +669,7 @@
     </row>
     <row r="3" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="str">
-        <f t="shared" ref="A3:A64" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
+        <f t="shared" ref="A3:A65" si="0">TEXT(ROW(A2),"0000")&amp;".jpg"</f>
         <v>0002.jpg</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1411,8 +1414,16 @@
       </c>
     </row>
     <row r="65" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="2"/>
-      <c r="C65" s="1"/>
+      <c r="A65" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0064.jpg</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="66" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2"/>

</xml_diff>